<commit_message>
Se actualiza la Base de datos
</commit_message>
<xml_diff>
--- a/Documents/Actividades realizadas/ActividadesN__.xlsx
+++ b/Documents/Actividades realizadas/ActividadesN__.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\1.- VioletaSystem\Documents\Actividades realizadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DDC944-032F-48EC-ADE9-ABD6600F64C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C411D5-6F1B-4FF3-AE0A-5B186204C330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="349">
   <si>
     <t>Descripción</t>
   </si>
@@ -1078,6 +1078,12 @@
   </si>
   <si>
     <t>Rediseño de filtros en la consulta de taller, estatus de taller, técnico del taller</t>
+  </si>
+  <si>
+    <t>Aprobación masiva en todos los tipos de estatus que tiene el taller desde la lista de talleres</t>
+  </si>
+  <si>
+    <t>Solución de problemas con la comilla simple en el código de barras</t>
   </si>
 </sst>
 </file>
@@ -1535,30 +1541,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="44" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1574,11 +1556,35 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="10" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1914,7 +1920,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K380"/>
+  <dimension ref="A1:K382"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -8449,229 +8455,249 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A338" s="5"/>
-      <c r="C338" s="61"/>
-      <c r="D338" s="13"/>
-      <c r="E338" s="2"/>
-      <c r="F338" s="2"/>
+      <c r="C338" s="61">
+        <v>46103</v>
+      </c>
+      <c r="D338" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="E338" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="F338" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="H338" s="14">
+        <v>3</v>
+      </c>
     </row>
     <row r="339" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A339" s="5"/>
-      <c r="C339" s="61"/>
-      <c r="D339" s="13"/>
-      <c r="E339" s="2"/>
-      <c r="F339" s="2"/>
+      <c r="C339" s="61">
+        <v>46103</v>
+      </c>
+      <c r="D339" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="E339" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F339" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="H339" s="14">
+        <v>2</v>
+      </c>
     </row>
     <row r="340" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A340" s="5"/>
+      <c r="C340" s="61"/>
+      <c r="D340" s="13"/>
       <c r="E340" s="2"/>
       <c r="F340" s="2"/>
     </row>
     <row r="341" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A341" s="75" t="s">
+      <c r="A341" s="5"/>
+      <c r="C341" s="61"/>
+      <c r="D341" s="13"/>
+      <c r="E341" s="2"/>
+      <c r="F341" s="2"/>
+    </row>
+    <row r="342" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A342" s="5"/>
+      <c r="E342" s="2"/>
+      <c r="F342" s="2"/>
+    </row>
+    <row r="343" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A343" s="83" t="s">
         <v>83</v>
       </c>
-      <c r="B341" s="75"/>
-      <c r="C341" s="75"/>
-      <c r="D341" s="75"/>
-      <c r="E341" s="75"/>
-      <c r="F341" s="75"/>
-      <c r="G341" s="16">
-        <f>SUM(G2:G340)</f>
+      <c r="B343" s="83"/>
+      <c r="C343" s="83"/>
+      <c r="D343" s="83"/>
+      <c r="E343" s="83"/>
+      <c r="F343" s="83"/>
+      <c r="G343" s="16">
+        <f>SUM(G2:G342)</f>
         <v>314.78999999999996</v>
       </c>
-      <c r="H341" s="16">
-        <f>SUM(H2:H340)</f>
-        <v>181.8</v>
-      </c>
-    </row>
-    <row r="342" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A342" s="75" t="s">
+      <c r="H343" s="16">
+        <f>SUM(H2:H342)</f>
+        <v>186.8</v>
+      </c>
+    </row>
+    <row r="344" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A344" s="83" t="s">
         <v>57</v>
       </c>
-      <c r="B342" s="75"/>
-      <c r="C342" s="75"/>
-      <c r="D342" s="75"/>
-      <c r="E342" s="75"/>
-      <c r="F342" s="75"/>
-      <c r="G342" s="16">
+      <c r="B344" s="83"/>
+      <c r="C344" s="83"/>
+      <c r="D344" s="83"/>
+      <c r="E344" s="83"/>
+      <c r="F344" s="83"/>
+      <c r="G344" s="16">
         <v>200</v>
       </c>
-      <c r="H342" s="16">
+      <c r="H344" s="16">
         <v>300</v>
       </c>
     </row>
-    <row r="343" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A343" s="75" t="s">
+    <row r="345" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A345" s="83" t="s">
         <v>84</v>
       </c>
-      <c r="B343" s="75"/>
-      <c r="C343" s="75"/>
-      <c r="D343" s="75"/>
-      <c r="E343" s="75"/>
-      <c r="F343" s="75"/>
-      <c r="G343" s="17">
-        <f>G342*G341</f>
-        <v>62957.999999999993</v>
-      </c>
-      <c r="H343" s="18">
-        <f>H342*H341</f>
-        <v>54540</v>
-      </c>
-      <c r="J343">
-        <v>-500</v>
-      </c>
-    </row>
-    <row r="344" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A344" s="75" t="s">
-        <v>58</v>
-      </c>
-      <c r="B344" s="75"/>
-      <c r="C344" s="75"/>
-      <c r="D344" s="75"/>
-      <c r="E344" s="75"/>
-      <c r="F344" s="75"/>
-      <c r="G344" s="80">
-        <f>G343+H343</f>
-        <v>117498</v>
-      </c>
-      <c r="H344" s="80"/>
-    </row>
-    <row r="345" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A345" s="10"/>
-      <c r="B345" s="83" t="s">
-        <v>60</v>
-      </c>
+      <c r="B345" s="83"/>
       <c r="C345" s="83"/>
       <c r="D345" s="83"/>
       <c r="E345" s="83"/>
       <c r="F345" s="83"/>
-      <c r="G345" s="21"/>
-    </row>
-    <row r="346" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A346" s="11">
-        <v>45109</v>
-      </c>
-      <c r="B346" s="84" t="s">
-        <v>59</v>
-      </c>
-      <c r="C346" s="84"/>
-      <c r="D346" s="84"/>
-      <c r="E346" s="84"/>
-      <c r="F346" s="84"/>
-      <c r="G346" s="85">
-        <v>10000</v>
-      </c>
-      <c r="H346" s="85"/>
+      <c r="G345" s="17">
+        <f>G344*G343</f>
+        <v>62957.999999999993</v>
+      </c>
+      <c r="H345" s="18">
+        <f>H344*H343</f>
+        <v>56040</v>
+      </c>
+      <c r="J345">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="346" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A346" s="83" t="s">
+        <v>58</v>
+      </c>
+      <c r="B346" s="83"/>
+      <c r="C346" s="83"/>
+      <c r="D346" s="83"/>
+      <c r="E346" s="83"/>
+      <c r="F346" s="83"/>
+      <c r="G346" s="72">
+        <f>G345+H345</f>
+        <v>118998</v>
+      </c>
+      <c r="H346" s="72"/>
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A347" s="11"/>
-      <c r="B347" s="86" t="s">
-        <v>96</v>
-      </c>
-      <c r="C347" s="86"/>
-      <c r="D347" s="86"/>
-      <c r="E347" s="86"/>
-      <c r="F347" s="86"/>
-      <c r="G347" s="85">
-        <v>5000</v>
-      </c>
-      <c r="H347" s="85"/>
+      <c r="A347" s="10"/>
+      <c r="B347" s="75" t="s">
+        <v>60</v>
+      </c>
+      <c r="C347" s="75"/>
+      <c r="D347" s="75"/>
+      <c r="E347" s="75"/>
+      <c r="F347" s="75"/>
+      <c r="G347" s="21"/>
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A348" s="11">
-        <v>45278</v>
+        <v>45109</v>
       </c>
       <c r="B348" s="76" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="C348" s="76"/>
       <c r="D348" s="76"/>
       <c r="E348" s="76"/>
       <c r="F348" s="76"/>
-      <c r="G348" s="85">
-        <v>9800</v>
-      </c>
-      <c r="H348" s="85"/>
+      <c r="G348" s="78">
+        <v>10000</v>
+      </c>
+      <c r="H348" s="78"/>
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A349" s="11"/>
-      <c r="B349" s="76"/>
-      <c r="C349" s="76"/>
-      <c r="D349" s="76"/>
-      <c r="E349" s="76"/>
-      <c r="F349" s="76"/>
-      <c r="G349" s="85">
-        <v>78298</v>
-      </c>
-      <c r="H349" s="85"/>
+      <c r="B349" s="79" t="s">
+        <v>96</v>
+      </c>
+      <c r="C349" s="79"/>
+      <c r="D349" s="79"/>
+      <c r="E349" s="79"/>
+      <c r="F349" s="79"/>
+      <c r="G349" s="78">
+        <v>5000</v>
+      </c>
+      <c r="H349" s="78"/>
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A350" s="11"/>
-      <c r="B350" s="76"/>
-      <c r="C350" s="76"/>
-      <c r="D350" s="76"/>
-      <c r="E350" s="76"/>
-      <c r="F350" s="76"/>
-      <c r="G350" s="85"/>
-      <c r="H350" s="85"/>
+      <c r="A350" s="11">
+        <v>45278</v>
+      </c>
+      <c r="B350" s="77" t="s">
+        <v>96</v>
+      </c>
+      <c r="C350" s="77"/>
+      <c r="D350" s="77"/>
+      <c r="E350" s="77"/>
+      <c r="F350" s="77"/>
+      <c r="G350" s="78">
+        <v>9800</v>
+      </c>
+      <c r="H350" s="78"/>
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A351" s="11"/>
-      <c r="B351" s="76"/>
-      <c r="C351" s="76"/>
-      <c r="D351" s="76"/>
-      <c r="E351" s="76"/>
-      <c r="F351" s="76"/>
-      <c r="G351" s="85"/>
-      <c r="H351" s="85"/>
+      <c r="B351" s="77"/>
+      <c r="C351" s="77"/>
+      <c r="D351" s="77"/>
+      <c r="E351" s="77"/>
+      <c r="F351" s="77"/>
+      <c r="G351" s="78">
+        <v>78298</v>
+      </c>
+      <c r="H351" s="78"/>
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A352" s="11"/>
-      <c r="B352" s="76" t="s">
-        <v>62</v>
-      </c>
-      <c r="C352" s="76"/>
-      <c r="D352" s="76"/>
-      <c r="E352" s="76"/>
-      <c r="F352" s="76"/>
-      <c r="G352" s="85">
-        <f>SUM(G346:H351)</f>
-        <v>103098</v>
-      </c>
-      <c r="H352" s="85"/>
-    </row>
-    <row r="353" spans="1:8" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A353" s="81" t="s">
-        <v>61</v>
-      </c>
-      <c r="B353" s="81"/>
-      <c r="C353" s="81"/>
-      <c r="D353" s="81"/>
-      <c r="E353" s="81"/>
-      <c r="F353" s="81"/>
-      <c r="G353" s="82">
-        <f>G344-G352</f>
-        <v>14400</v>
-      </c>
-      <c r="H353" s="82"/>
+      <c r="B352" s="77"/>
+      <c r="C352" s="77"/>
+      <c r="D352" s="77"/>
+      <c r="E352" s="77"/>
+      <c r="F352" s="77"/>
+      <c r="G352" s="78"/>
+      <c r="H352" s="78"/>
+    </row>
+    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A353" s="11"/>
+      <c r="B353" s="77"/>
+      <c r="C353" s="77"/>
+      <c r="D353" s="77"/>
+      <c r="E353" s="77"/>
+      <c r="F353" s="77"/>
+      <c r="G353" s="78"/>
+      <c r="H353" s="78"/>
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A354" s="11"/>
-      <c r="B354" s="12"/>
-      <c r="C354" s="12"/>
-      <c r="D354" s="12"/>
-      <c r="E354" s="12"/>
-      <c r="F354" s="12"/>
-    </row>
-    <row r="355" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A355" s="11"/>
-      <c r="B355" s="12"/>
-      <c r="C355" s="12"/>
-      <c r="D355" s="12"/>
-      <c r="E355" s="12"/>
-      <c r="F355" s="12"/>
+      <c r="B354" s="77" t="s">
+        <v>62</v>
+      </c>
+      <c r="C354" s="77"/>
+      <c r="D354" s="77"/>
+      <c r="E354" s="77"/>
+      <c r="F354" s="77"/>
+      <c r="G354" s="78">
+        <f>SUM(G348:H353)</f>
+        <v>103098</v>
+      </c>
+      <c r="H354" s="78"/>
+    </row>
+    <row r="355" spans="1:8" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="A355" s="73" t="s">
+        <v>61</v>
+      </c>
+      <c r="B355" s="73"/>
+      <c r="C355" s="73"/>
+      <c r="D355" s="73"/>
+      <c r="E355" s="73"/>
+      <c r="F355" s="73"/>
+      <c r="G355" s="74">
+        <f>G346-G354</f>
+        <v>15900</v>
+      </c>
+      <c r="H355" s="74"/>
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A356" s="11"/>
@@ -8802,190 +8828,206 @@
       <c r="F371" s="12"/>
     </row>
     <row r="372" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A372" s="9"/>
-      <c r="B372" s="77" t="s">
+      <c r="A372" s="11"/>
+      <c r="B372" s="12"/>
+      <c r="C372" s="12"/>
+      <c r="D372" s="12"/>
+      <c r="E372" s="12"/>
+      <c r="F372" s="12"/>
+    </row>
+    <row r="373" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A373" s="11"/>
+      <c r="B373" s="12"/>
+      <c r="C373" s="12"/>
+      <c r="D373" s="12"/>
+      <c r="E373" s="12"/>
+      <c r="F373" s="12"/>
+    </row>
+    <row r="374" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A374" s="9"/>
+      <c r="B374" s="84" t="s">
         <v>56</v>
       </c>
-      <c r="C372" s="77"/>
-      <c r="D372" s="77"/>
-      <c r="E372" s="77"/>
-      <c r="F372" s="77"/>
-      <c r="G372" s="20"/>
-      <c r="H372" s="20"/>
-      <c r="I372" s="7">
-        <f>G341+H341</f>
-        <v>496.59</v>
-      </c>
-      <c r="J372" s="7">
-        <f>I372</f>
-        <v>496.59</v>
-      </c>
-    </row>
-    <row r="373" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A373" s="5"/>
-      <c r="B373" s="78" t="s">
+      <c r="C374" s="84"/>
+      <c r="D374" s="84"/>
+      <c r="E374" s="84"/>
+      <c r="F374" s="84"/>
+      <c r="G374" s="20"/>
+      <c r="H374" s="20"/>
+      <c r="I374" s="7">
+        <f>G343+H343</f>
+        <v>501.59</v>
+      </c>
+      <c r="J374" s="7">
+        <f>I374</f>
+        <v>501.59</v>
+      </c>
+    </row>
+    <row r="375" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A375" s="5"/>
+      <c r="B375" s="85" t="s">
         <v>57</v>
       </c>
-      <c r="C373" s="78"/>
-      <c r="D373" s="78"/>
-      <c r="E373" s="78"/>
-      <c r="F373" s="78"/>
-      <c r="I373" s="7">
+      <c r="C375" s="85"/>
+      <c r="D375" s="85"/>
+      <c r="E375" s="85"/>
+      <c r="F375" s="85"/>
+      <c r="I375" s="7">
         <v>300</v>
       </c>
-      <c r="J373" s="7">
+      <c r="J375" s="7">
         <v>200</v>
       </c>
     </row>
-    <row r="374" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A374" s="5"/>
-      <c r="B374" s="78" t="s">
+    <row r="376" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A376" s="5"/>
+      <c r="B376" s="85" t="s">
         <v>58</v>
       </c>
-      <c r="C374" s="78"/>
-      <c r="D374" s="78"/>
-      <c r="E374" s="78"/>
-      <c r="F374" s="78"/>
-      <c r="I374" s="8">
-        <f>I373*I372</f>
-        <v>148977</v>
-      </c>
-      <c r="J374" s="8">
-        <f>J373*J372</f>
-        <v>99318</v>
-      </c>
-    </row>
-    <row r="375" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A375" s="22"/>
-      <c r="B375" s="79" t="s">
+      <c r="C376" s="85"/>
+      <c r="D376" s="85"/>
+      <c r="E376" s="85"/>
+      <c r="F376" s="85"/>
+      <c r="I376" s="8">
+        <f>I375*I374</f>
+        <v>150477</v>
+      </c>
+      <c r="J376" s="8">
+        <f>J375*J374</f>
+        <v>100318</v>
+      </c>
+    </row>
+    <row r="377" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A377" s="22"/>
+      <c r="B377" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="C375" s="79"/>
-      <c r="D375" s="79"/>
-      <c r="E375" s="79"/>
-      <c r="F375" s="79"/>
-      <c r="G375" s="23"/>
-      <c r="H375" s="23"/>
-      <c r="I375" s="24"/>
-      <c r="J375" s="24"/>
-    </row>
-    <row r="376" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A376" s="25">
+      <c r="C377" s="86"/>
+      <c r="D377" s="86"/>
+      <c r="E377" s="86"/>
+      <c r="F377" s="86"/>
+      <c r="G377" s="23"/>
+      <c r="H377" s="23"/>
+      <c r="I377" s="24"/>
+      <c r="J377" s="24"/>
+    </row>
+    <row r="378" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A378" s="25">
         <v>45109</v>
       </c>
-      <c r="B376" s="73" t="s">
+      <c r="B378" s="81" t="s">
         <v>59</v>
       </c>
-      <c r="C376" s="73"/>
-      <c r="D376" s="73"/>
-      <c r="E376" s="73"/>
-      <c r="F376" s="73"/>
-      <c r="G376" s="26"/>
-      <c r="H376" s="26"/>
-      <c r="I376" s="27">
-        <v>10000</v>
-      </c>
-      <c r="J376" s="27">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="377" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A377" s="25"/>
-      <c r="B377" s="28"/>
-      <c r="C377" s="28"/>
-      <c r="D377" s="28"/>
-      <c r="E377" s="28"/>
-      <c r="F377" s="28"/>
-      <c r="G377" s="26"/>
-      <c r="H377" s="26"/>
-      <c r="I377" s="29"/>
-      <c r="J377" s="29"/>
-    </row>
-    <row r="378" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A378" s="25"/>
-      <c r="B378" s="28"/>
-      <c r="C378" s="28"/>
-      <c r="D378" s="28"/>
-      <c r="E378" s="28"/>
-      <c r="F378" s="28"/>
+      <c r="C378" s="81"/>
+      <c r="D378" s="81"/>
+      <c r="E378" s="81"/>
+      <c r="F378" s="81"/>
       <c r="G378" s="26"/>
       <c r="H378" s="26"/>
-      <c r="I378" s="29"/>
-      <c r="J378" s="29"/>
-    </row>
-    <row r="379" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="I378" s="27">
+        <v>10000</v>
+      </c>
+      <c r="J378" s="27">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="379" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A379" s="25"/>
-      <c r="B379" s="74" t="s">
-        <v>62</v>
-      </c>
-      <c r="C379" s="74"/>
-      <c r="D379" s="74"/>
-      <c r="E379" s="74"/>
-      <c r="F379" s="74"/>
+      <c r="B379" s="28"/>
+      <c r="C379" s="28"/>
+      <c r="D379" s="28"/>
+      <c r="E379" s="28"/>
+      <c r="F379" s="28"/>
       <c r="G379" s="26"/>
       <c r="H379" s="26"/>
-      <c r="I379" s="30">
-        <f>SUM(I376:I378)</f>
+      <c r="I379" s="29"/>
+      <c r="J379" s="29"/>
+    </row>
+    <row r="380" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A380" s="25"/>
+      <c r="B380" s="28"/>
+      <c r="C380" s="28"/>
+      <c r="D380" s="28"/>
+      <c r="E380" s="28"/>
+      <c r="F380" s="28"/>
+      <c r="G380" s="26"/>
+      <c r="H380" s="26"/>
+      <c r="I380" s="29"/>
+      <c r="J380" s="29"/>
+    </row>
+    <row r="381" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A381" s="25"/>
+      <c r="B381" s="82" t="s">
+        <v>62</v>
+      </c>
+      <c r="C381" s="82"/>
+      <c r="D381" s="82"/>
+      <c r="E381" s="82"/>
+      <c r="F381" s="82"/>
+      <c r="G381" s="26"/>
+      <c r="H381" s="26"/>
+      <c r="I381" s="30">
+        <f>SUM(I378:I380)</f>
         <v>10000</v>
       </c>
-      <c r="J379" s="30">
-        <f>SUM(J376:J378)</f>
+      <c r="J381" s="30">
+        <f>SUM(J378:J380)</f>
         <v>10000</v>
       </c>
     </row>
-    <row r="380" spans="1:10" ht="33.75" x14ac:dyDescent="0.5">
-      <c r="A380" s="31">
+    <row r="382" spans="1:10" ht="33.75" x14ac:dyDescent="0.5">
+      <c r="A382" s="31">
         <v>45109</v>
       </c>
-      <c r="B380" s="72" t="s">
+      <c r="B382" s="80" t="s">
         <v>61</v>
       </c>
-      <c r="C380" s="72"/>
-      <c r="D380" s="72"/>
-      <c r="E380" s="72"/>
-      <c r="F380" s="72"/>
-      <c r="G380" s="32"/>
-      <c r="H380" s="32"/>
-      <c r="I380" s="33">
-        <f>I374-I379</f>
-        <v>138977</v>
-      </c>
-      <c r="J380" s="33">
-        <f>J374-J379</f>
-        <v>89318</v>
+      <c r="C382" s="80"/>
+      <c r="D382" s="80"/>
+      <c r="E382" s="80"/>
+      <c r="F382" s="80"/>
+      <c r="G382" s="32"/>
+      <c r="H382" s="32"/>
+      <c r="I382" s="33">
+        <f>I376-I381</f>
+        <v>140477</v>
+      </c>
+      <c r="J382" s="33">
+        <f>J376-J381</f>
+        <v>90318</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="G344:H344"/>
-    <mergeCell ref="A353:F353"/>
-    <mergeCell ref="G353:H353"/>
-    <mergeCell ref="B345:F345"/>
-    <mergeCell ref="B346:F346"/>
+    <mergeCell ref="B382:F382"/>
+    <mergeCell ref="B378:F378"/>
+    <mergeCell ref="B381:F381"/>
+    <mergeCell ref="A344:F344"/>
+    <mergeCell ref="A343:F343"/>
+    <mergeCell ref="A345:F345"/>
+    <mergeCell ref="A346:F346"/>
     <mergeCell ref="B352:F352"/>
-    <mergeCell ref="G346:H346"/>
-    <mergeCell ref="G347:H347"/>
-    <mergeCell ref="G352:H352"/>
-    <mergeCell ref="G349:H349"/>
-    <mergeCell ref="G350:H350"/>
-    <mergeCell ref="G351:H351"/>
-    <mergeCell ref="G348:H348"/>
-    <mergeCell ref="B348:F348"/>
-    <mergeCell ref="B347:F347"/>
-    <mergeCell ref="B349:F349"/>
-    <mergeCell ref="B380:F380"/>
-    <mergeCell ref="B376:F376"/>
-    <mergeCell ref="B379:F379"/>
-    <mergeCell ref="A342:F342"/>
-    <mergeCell ref="A341:F341"/>
-    <mergeCell ref="A343:F343"/>
-    <mergeCell ref="A344:F344"/>
-    <mergeCell ref="B350:F350"/>
-    <mergeCell ref="B351:F351"/>
-    <mergeCell ref="B372:F372"/>
-    <mergeCell ref="B373:F373"/>
+    <mergeCell ref="B353:F353"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B375:F375"/>
+    <mergeCell ref="B376:F376"/>
+    <mergeCell ref="B377:F377"/>
+    <mergeCell ref="G346:H346"/>
+    <mergeCell ref="A355:F355"/>
+    <mergeCell ref="G355:H355"/>
+    <mergeCell ref="B347:F347"/>
+    <mergeCell ref="B348:F348"/>
+    <mergeCell ref="B354:F354"/>
+    <mergeCell ref="G348:H348"/>
+    <mergeCell ref="G349:H349"/>
+    <mergeCell ref="G354:H354"/>
+    <mergeCell ref="G351:H351"/>
+    <mergeCell ref="G352:H352"/>
+    <mergeCell ref="G353:H353"/>
+    <mergeCell ref="G350:H350"/>
+    <mergeCell ref="B350:F350"/>
+    <mergeCell ref="B349:F349"/>
+    <mergeCell ref="B351:F351"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>